<commit_message>
column header change in Devices template
</commit_message>
<xml_diff>
--- a/api/templates/export/devices/en.xlsx
+++ b/api/templates/export/devices/en.xlsx
@@ -5,11 +5,11 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\devices\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-node-12\api\templates\export\devices\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815"/>
+    <workbookView xWindow="480" yWindow="480" windowWidth="20736" windowHeight="11760" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
@@ -183,16 +183,16 @@
     <t>Last Seen On</t>
   </si>
   <si>
-    <t>Error Rate</t>
-  </si>
-  <si>
-    <t>Availability</t>
-  </si>
-  <si>
     <t># Last Month</t>
   </si>
   <si>
     <t># This Month</t>
+  </si>
+  <si>
+    <t>% Active</t>
+  </si>
+  <si>
+    <t>% Test Failures</t>
   </si>
 </sst>
 </file>
@@ -840,42 +840,42 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35.5" style="9" customWidth="1"/>
-    <col min="2" max="2" width="23.125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.625" style="15" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.59765625" style="15" customWidth="1"/>
     <col min="4" max="4" width="11.5" style="15" customWidth="1"/>
-    <col min="5" max="5" width="28.625" style="3" customWidth="1"/>
-    <col min="6" max="6" width="20.75" style="3" customWidth="1"/>
+    <col min="5" max="5" width="28.59765625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="20.69921875" style="3" customWidth="1"/>
     <col min="7" max="7" width="20" style="3" customWidth="1"/>
-    <col min="8" max="8" width="18.75" style="3" customWidth="1"/>
+    <col min="8" max="8" width="18.69921875" style="3" customWidth="1"/>
     <col min="9" max="9" width="18" style="3" customWidth="1"/>
-    <col min="10" max="10" width="16.375" style="3" customWidth="1"/>
+    <col min="10" max="10" width="16.3984375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
     </row>
-    <row r="3" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C3" s="15"/>
       <c r="D3" s="15"/>
     </row>
-    <row r="4" spans="1:10" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>33</v>
       </c>
@@ -883,10 +883,10 @@
         <v>34</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>44</v>
@@ -901,13 +901,13 @@
         <v>51</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
@@ -939,7 +939,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="8"/>
@@ -958,14 +958,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
+    <col min="1" max="1" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.19921875" customWidth="1"/>
+    <col min="3" max="3" width="100.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -976,7 +976,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>1001</v>
       </c>
@@ -987,7 +987,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <v>1002</v>
       </c>
@@ -998,7 +998,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>1004</v>
       </c>
@@ -1009,7 +1009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>1005</v>
       </c>
@@ -1020,7 +1020,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>1006</v>
       </c>
@@ -1031,7 +1031,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1007</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>1017</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>1018</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>2003</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>2005</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>2008</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>2009</v>
       </c>
@@ -1108,7 +1108,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>2011</v>
       </c>
@@ -1119,7 +1119,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>2014</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>2016</v>
       </c>
@@ -1141,7 +1141,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>2018</v>
       </c>
@@ -1152,7 +1152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>2022</v>
       </c>
@@ -1163,7 +1163,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>2025</v>
       </c>
@@ -1174,7 +1174,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <v>2032</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>2034</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>2037</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>4010</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
         <v>4017</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>5006</v>
       </c>
@@ -1240,7 +1240,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5">
         <v>5007</v>
       </c>
@@ -1251,7 +1251,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
make Excel headers fully match web pages
</commit_message>
<xml_diff>
--- a/api/templates/export/devices/en.xlsx
+++ b/api/templates/export/devices/en.xlsx
@@ -5,7 +5,7 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-node-12\api\templates\export\devices\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\devices\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -126,9 +126,6 @@
     <t>Signal loss detected in the amplification curve</t>
   </si>
   <si>
-    <t>Device Name</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
@@ -180,19 +177,22 @@
     <t>Printed on &lt;date&gt;</t>
   </si>
   <si>
-    <t>Last Seen On</t>
-  </si>
-  <si>
-    <t># Last Month</t>
-  </si>
-  <si>
-    <t># This Month</t>
-  </si>
-  <si>
-    <t>% Active</t>
-  </si>
-  <si>
-    <t>% Test Failures</t>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Test Failures</t>
+  </si>
+  <si>
+    <t>Last Seen</t>
+  </si>
+  <si>
+    <t>Last Month</t>
+  </si>
+  <si>
+    <t>This Month</t>
   </si>
 </sst>
 </file>
@@ -856,12 +856,12 @@
   <sheetData>
     <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C2" s="15"/>
       <c r="D2" s="15"/>
@@ -872,71 +872,71 @@
     </row>
     <row r="4" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:10" s="6" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="C5" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="J5" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>36</v>
-      </c>
       <c r="C6" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="E6" s="13" t="s">
-        <v>48</v>
-      </c>
       <c r="F6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>39</v>
-      </c>
       <c r="I6" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
- Removed duplicated fields from device list query - Showing lastPingOn as the Last Seen column in device list export (matching now with the UI list)
</commit_message>
<xml_diff>
--- a/api/templates/export/devices/en.xlsx
+++ b/api/templates/export/devices/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25831"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\export\devices\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\export\devices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227B54E0-E37C-41F2-8864-DB61C893A270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CAC13A-F543-4CCE-8344-2200F7B98383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
@@ -42,9 +42,6 @@
     <t>&lt;createdOn&gt;</t>
   </si>
   <si>
-    <t>&lt;lastSeen&gt;</t>
-  </si>
-  <si>
     <t>Aspect Devices</t>
   </si>
   <si>
@@ -94,6 +91,9 @@
   </si>
   <si>
     <t>This Month</t>
+  </si>
+  <si>
+    <t>&lt;lastPingOn&gt;</t>
   </si>
 </sst>
 </file>
@@ -737,7 +737,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="35.5" style="7" customWidth="1"/>
     <col min="2" max="2" width="23.09765625" style="2" customWidth="1"/>
@@ -751,60 +751,60 @@
     <col min="10" max="10" width="16.3984375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="20.399999999999999" x14ac:dyDescent="0.75">
       <c r="A1" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.6">
       <c r="A2" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
     </row>
-    <row r="3" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.6">
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" ht="15.9" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A4" s="7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:10" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A5" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="12" t="s">
-        <v>19</v>
-      </c>
       <c r="E5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>22</v>
-      </c>
     </row>
-    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.6">
       <c r="A6" s="10" t="s">
         <v>1</v>
       </c>
@@ -812,31 +812,31 @@
         <v>2</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.6">
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
       <c r="E8" s="6"/>

</xml_diff>

<commit_message>
[feat/ASP-8050-Add-Notes-fields-to-Device-List-Download] Added Notes field to Device List Download
</commit_message>
<xml_diff>
--- a/api/templates/export/devices/en.xlsx
+++ b/api/templates/export/devices/en.xlsx
@@ -1,118 +1,113 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25831"/>
-  <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\export\devices\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CAC13A-F543-4CCE-8344-2200F7B98383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10531"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8D5C93A-EB9F-7144-9443-E1E12A93E21A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>Aspect Devices</t>
+  </si>
+  <si>
+    <t>Printed on &lt;date&gt;</t>
+  </si>
+  <si>
+    <t>&lt;Table&gt;</t>
+  </si>
+  <si>
+    <t>Device</t>
+  </si>
   <si>
     <t>Status</t>
   </si>
   <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Test Failures</t>
+  </si>
+  <si>
+    <t>Issues</t>
+  </si>
+  <si>
+    <t>Reporting Since</t>
+  </si>
+  <si>
+    <t>Short name</t>
+  </si>
+  <si>
+    <t>Last Seen</t>
+  </si>
+  <si>
+    <t>Last Month</t>
+  </si>
+  <si>
+    <t>This Month</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
     <t>&lt;name&gt;</t>
   </si>
   <si>
     <t>&lt;status&gt;</t>
   </si>
   <si>
-    <t>Reporting Since</t>
+    <t>&lt;availabilityRate&gt;</t>
+  </si>
+  <si>
+    <t>&lt;errorRate&gt;</t>
+  </si>
+  <si>
+    <t>&lt;issuesCategories&gt;</t>
   </si>
   <si>
     <t>&lt;createdOn&gt;</t>
   </si>
   <si>
-    <t>Aspect Devices</t>
-  </si>
-  <si>
-    <t>Short name</t>
-  </si>
-  <si>
     <t>&lt;shortName&gt;</t>
   </si>
   <si>
-    <t>&lt;availabilityRate&gt;</t>
-  </si>
-  <si>
-    <t>Issues</t>
+    <t>&lt;lastPingOn&gt;</t>
+  </si>
+  <si>
+    <t>&lt;resultCountLastMonth&gt;</t>
   </si>
   <si>
     <t>&lt;resultCountThisMonth&gt;</t>
   </si>
   <si>
-    <t>&lt;resultCountLastMonth&gt;</t>
-  </si>
-  <si>
-    <t>&lt;errorRate&gt;</t>
-  </si>
-  <si>
-    <t>&lt;issuesCategories&gt;</t>
-  </si>
-  <si>
-    <t>&lt;Table&gt;</t>
-  </si>
-  <si>
-    <t>Printed on &lt;date&gt;</t>
-  </si>
-  <si>
-    <t>Device</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Test Failures</t>
-  </si>
-  <si>
-    <t>Last Seen</t>
-  </si>
-  <si>
-    <t>Last Month</t>
-  </si>
-  <si>
-    <t>This Month</t>
-  </si>
-  <si>
-    <t>&lt;lastPingOn&gt;</t>
+    <t>&lt;notes&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -128,17 +123,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="12"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -166,7 +153,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -205,6 +192,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color auto="1"/>
       </left>
@@ -235,174 +237,68 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
-  <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD7D7D7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
-  <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
-    </tableStyle>
-  </tableStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -736,118 +632,120 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="35.5" style="7" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="12.59765625" style="13" customWidth="1"/>
-    <col min="4" max="4" width="11.5" style="13" customWidth="1"/>
-    <col min="5" max="5" width="28.59765625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.69921875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="35.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="3" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="2" customWidth="1"/>
     <col min="7" max="7" width="20" style="2" customWidth="1"/>
-    <col min="8" max="8" width="18.69921875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="18.6640625" style="2" customWidth="1"/>
     <col min="9" max="9" width="18" style="2" customWidth="1"/>
-    <col min="10" max="10" width="16.3984375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="16.33203125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.399999999999999" x14ac:dyDescent="0.75">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:11" ht="20.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:11" s="1" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" s="5" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>5</v>
       </c>
+      <c r="D5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="7" t="s">
+    <row r="6" spans="1:11" s="2" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
+      <c r="C6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" s="7" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:10" ht="15.9" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
-      <c r="E8" s="6"/>
+      <c r="E8" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
-  <extLst>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
-      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
-    </ext>
-  </extLst>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967292" verticalDpi="4294967292"/>
 </worksheet>
 </file>
</xml_diff>